<commit_message>
feat: update template_import_cadastral.xlsx for improved data import functionality
</commit_message>
<xml_diff>
--- a/lead-import-visualizer/public/templates/template_import_cadastral.xlsx
+++ b/lead-import-visualizer/public/templates/template_import_cadastral.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pichau\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{646A36F4-6DE9-4FB5-A003-A9489D81AAD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C76E7789-C3FF-47CD-905E-EEF6ED1C4B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="690" yWindow="2460" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>CpfCliente</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>NomeCliente</t>
+  </si>
+  <si>
+    <t>Vendedor</t>
   </si>
 </sst>
 </file>
@@ -473,7 +476,7 @@
     <col min="13" max="13" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -510,50 +513,53 @@
       <c r="L1" s="6" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L2" s="1"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L4" s="1"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L5" s="1"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L6" s="1"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L7" s="1"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L8" s="1"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L9" s="1"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L10" s="1"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L11" s="1"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L12" s="1"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L13" s="1"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L14" s="1"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L15" s="1"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L16" s="1"/>
     </row>
     <row r="17" spans="9:12" x14ac:dyDescent="0.25">

</xml_diff>